<commit_message>
Refresh state-wise overdue data from praapti.in (as of 2026-08-06)
Re-scraped home/getStateWiseOverdueReport. National totals now:
Current 63,071.9 Cr, Overdue Before Trigger 21,995.4 Cr,
Overdue After Trigger 4.3 Cr (portal last updated 2026-08-04).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QDkN6JmvLtVVBxV7MZ6VWz
</commit_message>
<xml_diff>
--- a/Praapti_StateWise_Overdue.xlsx
+++ b/Praapti_StateWise_Overdue.xlsx
@@ -528,7 +528,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: https://praapti.in (home/getStateWiseOverdueReport)  |  All amounts in Rs. Crore  |  Scraped: 2026-07-07</t>
+          <t>Source: https://praapti.in (home/getStateWiseOverdueReport)  |  All amounts in Rs. Crore  |  Scraped: 2026-08-06</t>
         </is>
       </c>
     </row>
@@ -610,16 +610,16 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>3040.4326862</v>
+        <v>3374.8435658</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>4683.8739946</v>
+        <v>2078.1672604</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>4683.8739946</v>
+        <v>2078.1672604</v>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
@@ -639,16 +639,16 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>54.5921456</v>
+        <v>46.5277632</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.0210185</v>
+        <v>0</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>0.0005735</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.021592</v>
+        <v>0.0005735</v>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
@@ -668,20 +668,20 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1338.2603332</v>
+        <v>1362.6104004</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>110.6199776</v>
+        <v>8.0749317</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.6698489</v>
+        <v>0</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>111.2898265</v>
-      </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>Overdue After Trigger Date</t>
+        <v>8.0749317</v>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Overdue Before Trigger Date</t>
         </is>
       </c>
     </row>
@@ -697,16 +697,16 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>2834.6216838</v>
+        <v>3839.0190263</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>215.5762238</v>
+        <v>498.2088889</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>215.5762238</v>
+        <v>498.2088889</v>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
@@ -726,16 +726,16 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>168.7950297</v>
+        <v>73.9443625</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>5.397361</v>
+        <v>0</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>0.0040492</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>5.4014102</v>
+        <v>0.0040492</v>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
@@ -755,16 +755,16 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>1696.7757483</v>
+        <v>1811.8020402</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>123.5373258</v>
+        <v>157.0040406</v>
       </c>
       <c r="E11" s="6" t="n">
         <v>0.047929</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>123.5852548</v>
+        <v>157.0519696</v>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
@@ -784,20 +784,20 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>384.2598354</v>
+        <v>690.7397883</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>0</v>
+        <v>34.0202683</v>
       </c>
       <c r="E12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>Current dues</t>
+        <v>34.0202683</v>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Overdue Before Trigger Date</t>
         </is>
       </c>
     </row>
@@ -813,16 +813,16 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>1627.0191655</v>
+        <v>1944.1923519</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>374.59719</v>
+        <v>102.6744663</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>0.830774</v>
+        <v>0.7539308</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>375.427964</v>
+        <v>103.4283971</v>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
@@ -842,16 +842,16 @@
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>176.979255</v>
+        <v>161.1198078</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>0.9449812</v>
+        <v>2.9224555</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>0.9449812</v>
+        <v>2.9224555</v>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
@@ -871,16 +871,16 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>2032.897577</v>
+        <v>1709.5637652</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>72.8045296</v>
+        <v>189.9644661</v>
       </c>
       <c r="E15" s="6" t="n">
         <v>9e-07</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>72.8045305</v>
+        <v>189.964467</v>
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
@@ -900,16 +900,16 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>3096.1058365</v>
+        <v>2805.3015206</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>857.6484569</v>
+        <v>498.2912905</v>
       </c>
       <c r="E16" s="6" t="n">
         <v>3e-07</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>857.6484572000001</v>
+        <v>498.2912908</v>
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
@@ -929,16 +929,16 @@
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>448.4796987</v>
+        <v>424.0632695</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>61.5654844</v>
+        <v>2.8531889</v>
       </c>
       <c r="E17" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>61.5654844</v>
+        <v>2.8531889</v>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
@@ -958,16 +958,16 @@
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1146.358937</v>
+        <v>1152.0384424</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>137.4653995</v>
+        <v>137.6310807</v>
       </c>
       <c r="E18" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>137.4653995</v>
+        <v>137.6310807</v>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
@@ -987,16 +987,16 @@
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>1393.1084868</v>
+        <v>1814.9107098</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>465.2024644</v>
+        <v>1017.7144886</v>
       </c>
       <c r="E19" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>465.2024644</v>
+        <v>1017.7144886</v>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
@@ -1016,16 +1016,16 @@
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>4208.6450532</v>
+        <v>4643.5388957</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>2676.8562635</v>
+        <v>2809.3217151</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>1.5014108</v>
+        <v>1.8119455</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>2678.3576743</v>
+        <v>2811.1336606</v>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
@@ -1045,16 +1045,16 @@
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>1196.5581023</v>
+        <v>1264.9326348</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>115.5689353</v>
+        <v>555.9339634</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>0.1243686</v>
+        <v>0.139633</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>115.6933039</v>
+        <v>556.0735964</v>
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
@@ -1103,16 +1103,16 @@
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>4244.5043499</v>
+        <v>4276.8176826</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>331.139619</v>
+        <v>902.0122104</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0.0164181</v>
+        <v>0.0172493</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>331.1560371</v>
+        <v>902.0294597</v>
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
@@ -1132,16 +1132,16 @@
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>6096.2395919</v>
+        <v>6020.3551336</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>3327.077775</v>
+        <v>1863.0093835</v>
       </c>
       <c r="E24" s="6" t="n">
         <v>0.5829442</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>3327.6607192</v>
+        <v>1863.5923277</v>
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
@@ -1161,20 +1161,20 @@
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>129.5316479</v>
+        <v>140.1241112</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>56.0643798</v>
+        <v>54.8666033</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>0.9658137</v>
+        <v>0</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>57.0301935</v>
-      </c>
-      <c r="G25" s="9" t="inlineStr">
-        <is>
-          <t>Overdue After Trigger Date</t>
+        <v>54.8666033</v>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Overdue Before Trigger Date</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>117.1909547</v>
+        <v>78.0945079</v>
       </c>
       <c r="D26" s="6" t="n">
         <v>0</v>
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>49.7079529</v>
+        <v>35.6164405</v>
       </c>
       <c r="D27" s="6" t="n">
         <v>0</v>
@@ -1248,20 +1248,20 @@
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>77.7161428</v>
+        <v>62.5113693</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>3.0652406</v>
+        <v>0</v>
       </c>
       <c r="E28" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>3.0652406</v>
-      </c>
-      <c r="G28" s="8" t="inlineStr">
-        <is>
-          <t>Overdue Before Trigger Date</t>
+        <v>0</v>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>Current dues</t>
         </is>
       </c>
     </row>
@@ -1277,16 +1277,16 @@
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>1465.4439027</v>
+        <v>1672.3764556</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>616.904196</v>
+        <v>392.7244689</v>
       </c>
       <c r="E29" s="6" t="n">
         <v>0.2621178</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>617.1663138</v>
+        <v>392.9865867</v>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
@@ -1306,7 +1306,7 @@
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>127.4399825</v>
+        <v>223.0331692</v>
       </c>
       <c r="D30" s="6" t="n">
         <v>0</v>
@@ -1335,16 +1335,16 @@
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>1857.9866925</v>
+        <v>2528.2792109</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>681.0290081000001</v>
+        <v>1072.5297172</v>
       </c>
       <c r="E31" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>681.0290081000001</v>
+        <v>1072.5297172</v>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
@@ -1364,16 +1364,16 @@
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>4153.2009399</v>
+        <v>4481.1058297</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>1584.6429554</v>
+        <v>1894.1654563</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>0.009858799999999999</v>
+        <v>0.0474065</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>1584.6528142</v>
+        <v>1894.2128628</v>
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
@@ -1393,16 +1393,16 @@
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>63.2797563</v>
+        <v>66.257171</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>28.5686513</v>
+        <v>2.7128798</v>
       </c>
       <c r="E33" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>28.5686513</v>
+        <v>2.7128798</v>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
@@ -1422,16 +1422,16 @@
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>4521.2696975</v>
+        <v>3719.5318507</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>619.9269015</v>
+        <v>678.6860172</v>
       </c>
       <c r="E34" s="6" t="n">
         <v>2e-07</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>619.9269017</v>
+        <v>678.6860174</v>
       </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
@@ -1451,16 +1451,16 @@
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>1789.1543569</v>
+        <v>1597.6646801</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>802.3674586</v>
+        <v>205.6241921</v>
       </c>
       <c r="E35" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>802.3674586</v>
+        <v>205.6241921</v>
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
@@ -1480,16 +1480,16 @@
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>270.4927356</v>
+        <v>320.3415829</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>171.8731148</v>
+        <v>154.7158621</v>
       </c>
       <c r="E36" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>171.8731148</v>
+        <v>154.7158621</v>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
@@ -1509,16 +1509,16 @@
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>7533.2900107</v>
+        <v>7883.0419084</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>5504.6599706</v>
+        <v>6385.140427</v>
       </c>
       <c r="E37" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>5504.6599706</v>
+        <v>6385.140427</v>
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
@@ -1538,16 +1538,16 @@
         </is>
       </c>
       <c r="C38" s="6" t="n">
-        <v>998.6295801</v>
+        <v>926.9452156999999</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>88.4202219</v>
+        <v>155.8781753</v>
       </c>
       <c r="E38" s="6" t="n">
         <v>0.2634166</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>88.6836385</v>
+        <v>156.1415919</v>
       </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
@@ -1567,16 +1567,16 @@
         </is>
       </c>
       <c r="C39" s="6" t="n">
-        <v>1821.9759019</v>
+        <v>1920.6624006</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>146.4435014</v>
+        <v>140.554156</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>0.3210671</v>
+        <v>0.3530568</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>146.7645685</v>
+        <v>140.9072128</v>
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
@@ -1592,16 +1592,16 @@
       </c>
       <c r="B40" s="12" t="n"/>
       <c r="C40" s="13" t="n">
-        <v>60160.9437709</v>
+        <v>63071.9070643</v>
       </c>
       <c r="D40" s="13" t="n">
-        <v>23863.8626001</v>
+        <v>21995.4020541</v>
       </c>
       <c r="E40" s="13" t="n">
-        <v>5.6005917</v>
+        <v>4.2842536</v>
       </c>
       <c r="F40" s="13" t="n">
-        <v>23869.4631918</v>
+        <v>21999.6863077</v>
       </c>
       <c r="G40" s="12" t="n"/>
     </row>

</xml_diff>

<commit_message>
Refresh state-wise overdue data from praapti.in (as of 2026-09-09)
Re-scraped home/getStateWiseOverdueReport. National totals now:
Current 64,049.4 Cr, Overdue Before Trigger 21,756.8 Cr,
Overdue After Trigger 4.9 Cr (portal last updated 2026-09-03).

Report now lists 33 states/UTs (down from 35): Andaman & Nicobar
Islands and Lakshadweep, both previously zero-value 'No Registered
Discom' entries, are no longer returned.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QDkN6JmvLtVVBxV7MZ6VWz
</commit_message>
<xml_diff>
--- a/Praapti_StateWise_Overdue.xlsx
+++ b/Praapti_StateWise_Overdue.xlsx
@@ -10,7 +10,7 @@
     <sheet name="State-wise Overdue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'State-wise Overdue'!$A$4:$G$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'State-wise Overdue'!$A$4:$G$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -46,7 +46,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -56,11 +56,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00312E81"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E0E0E0"/>
       </patternFill>
     </fill>
     <fill>
@@ -110,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -133,12 +128,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -506,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -528,7 +520,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: https://praapti.in (home/getStateWiseOverdueReport)  |  All amounts in Rs. Crore  |  Scraped: 2026-08-06</t>
+          <t>Source: https://praapti.in (home/getStateWiseOverdueReport)  |  All amounts in Rs. Crore  |  Scraped: 2026-09-09</t>
         </is>
       </c>
     </row>
@@ -572,85 +564,85 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Andaman and Nicobar Islands</t>
+          <t>Andhra Pradesh</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>ANI</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0</v>
+        <v>3361.3710722</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0</v>
+        <v>2709.6378901</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0</v>
+        <v>2709.6378901</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>No Registered Discom</t>
+          <t>Overdue Before Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Andhra Pradesh</t>
+          <t>Arunachal Pradesh</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>ACP</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>3374.8435658</v>
+        <v>47.8955964</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2078.1672604</v>
+        <v>0.6029133</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0</v>
+        <v>0.0005735</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>2078.1672604</v>
+        <v>0.6034868</v>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Overdue Before Trigger Date</t>
+          <t>Overdue After Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Arunachal Pradesh</t>
+          <t>Assam</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>ACP</t>
+          <t>ASM</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>46.5277632</v>
+        <v>1360.5232556</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0</v>
+        <v>35.7164126</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.0005735</v>
+        <v>0.4617117</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.0005735</v>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
+        <v>36.1781243</v>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>Overdue After Trigger Date</t>
         </is>
@@ -659,85 +651,85 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Assam</t>
+          <t>Bihar</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>ASM</t>
+          <t>BHR</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1362.6104004</v>
+        <v>3887.1073671</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>8.0749317</v>
+        <v>727.6239772</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0</v>
+        <v>0.1536194</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>8.0749317</v>
+        <v>727.7775966</v>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>Overdue Before Trigger Date</t>
+          <t>Overdue After Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Bihar</t>
+          <t>Chandigarh</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>BHR</t>
+          <t>CHG</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>3839.0190263</v>
+        <v>201.2615955</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>498.2088889</v>
+        <v>5.0556505</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0</v>
+        <v>0.0040492</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>498.2088889</v>
+        <v>5.0596997</v>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>Overdue Before Trigger Date</t>
+          <t>Overdue After Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Chandigarh</t>
+          <t>Chhattisgarh</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>CHG</t>
+          <t>CTG</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>73.9443625</v>
+        <v>2268.8155338</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0</v>
+        <v>66.2599251</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.0040492</v>
+        <v>0.047929</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.0040492</v>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
+        <v>66.3078541</v>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
         <is>
           <t>Overdue After Trigger Date</t>
         </is>
@@ -746,143 +738,143 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Chhattisgarh</t>
+          <t>DNH &amp; DD</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>CTG</t>
+          <t>DNH</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>1811.8020402</v>
+        <v>729.3385638</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>157.0040406</v>
+        <v>1.7721306</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.047929</v>
+        <v>0</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>157.0519696</v>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>Overdue After Trigger Date</t>
+        <v>1.7721306</v>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Overdue Before Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>DNH &amp; DD</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>DNH</t>
+          <t>DL</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>690.7397883</v>
+        <v>1814.746618</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>34.0202683</v>
+        <v>117.5293895</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>0</v>
+        <v>0.7150193</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>34.0202683</v>
+        <v>118.2444088</v>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Overdue Before Trigger Date</t>
+          <t>Overdue After Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Goa</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>DL</t>
+          <t>GOA</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>1944.1923519</v>
+        <v>87.06176550000001</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>102.6744663</v>
+        <v>1.0048546</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>0.7539308</v>
+        <v>0</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>103.4283971</v>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>Overdue After Trigger Date</t>
+        <v>1.0048546</v>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Overdue Before Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Goa</t>
+          <t>Gujarat</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>GOA</t>
+          <t>GJT</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>161.1198078</v>
+        <v>2884.7720937</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>2.9224555</v>
+        <v>119.8052713</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>0</v>
+        <v>9e-07</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>2.9224555</v>
+        <v>119.8052722</v>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Overdue Before Trigger Date</t>
+          <t>Overdue After Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Gujarat</t>
+          <t>Haryana</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>GJT</t>
+          <t>HRN</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>1709.5637652</v>
+        <v>3382.6870038</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>189.9644661</v>
+        <v>1410.8557868</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>9e-07</v>
+        <v>3e-07</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>189.964467</v>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
+        <v>1410.8557871</v>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>Overdue After Trigger Date</t>
         </is>
@@ -891,85 +883,85 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Haryana</t>
+          <t>Himachal Pradesh</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>HRN</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>2805.3015206</v>
+        <v>423.7210428</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>498.2912905</v>
+        <v>36.4218143</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>3e-07</v>
+        <v>0</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>498.2912908</v>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>Overdue After Trigger Date</t>
+        <v>36.4218143</v>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Overdue Before Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Himachal Pradesh</t>
+          <t>Jammu and Kashmir</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>JAK</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>424.0632695</v>
+        <v>1307.5120904</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>2.8531889</v>
+        <v>0</v>
       </c>
       <c r="E17" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>2.8531889</v>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>Overdue Before Trigger Date</t>
+        <v>0</v>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>Current dues</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Jammu and Kashmir</t>
+          <t>Jharkhand</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>JAK</t>
+          <t>JHK</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1152.0384424</v>
+        <v>1987.785782</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>137.6310807</v>
+        <v>30.9451448</v>
       </c>
       <c r="E18" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>137.6310807</v>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
+        <v>30.9451448</v>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>Overdue Before Trigger Date</t>
         </is>
@@ -978,56 +970,56 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Jharkhand</t>
+          <t>Karnataka</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>JHK</t>
+          <t>KRT</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>1814.9107098</v>
+        <v>4847.3128162</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>1017.7144886</v>
+        <v>2801.3576706</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>0</v>
+        <v>1.8787265</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>1017.7144886</v>
+        <v>2803.2363971</v>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Overdue Before Trigger Date</t>
+          <t>Overdue After Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Karnataka</t>
+          <t>Kerala</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>KRT</t>
+          <t>KRL</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>4643.5388957</v>
+        <v>773.3769996</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>2809.3217151</v>
+        <v>32.9250338</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>1.8119455</v>
+        <v>0.1701943</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>2811.1336606</v>
-      </c>
-      <c r="G20" s="9" t="inlineStr">
+        <v>33.0952281</v>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>Overdue After Trigger Date</t>
         </is>
@@ -1036,27 +1028,27 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Kerala</t>
+          <t>Madhya Pradesh</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>KRL</t>
+          <t>MPD</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>1264.9326348</v>
+        <v>2976.5197561</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>555.9339634</v>
+        <v>865.6462972</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>0.139633</v>
+        <v>0.0178909</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>556.0735964</v>
-      </c>
-      <c r="G21" s="9" t="inlineStr">
+        <v>865.6641881</v>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>Overdue After Trigger Date</t>
         </is>
@@ -1065,132 +1057,132 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Lakshadweep</t>
+          <t>Maharashtra</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>MHA</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>0</v>
+        <v>6161.2741929</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>0</v>
+        <v>2298.2043696</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>0</v>
+        <v>0.5829442</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>No Registered Discom</t>
+        <v>2298.7873138</v>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Overdue After Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Madhya Pradesh</t>
+          <t>Manipur</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>MPD</t>
+          <t>MIP</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>4276.8176826</v>
+        <v>145.051854</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>902.0122104</v>
+        <v>42.151892</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0.0172493</v>
+        <v>0</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>902.0294597</v>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>Overdue After Trigger Date</t>
+        <v>42.151892</v>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Overdue Before Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Maharashtra</t>
+          <t>Meghalaya</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>MHA</t>
+          <t>MGA</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>6020.3551336</v>
+        <v>80.4057152</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>1863.0093835</v>
+        <v>2.9477522</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>0.5829442</v>
+        <v>0</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>1863.5923277</v>
-      </c>
-      <c r="G24" s="9" t="inlineStr">
-        <is>
-          <t>Overdue After Trigger Date</t>
+        <v>2.9477522</v>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Overdue Before Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Manipur</t>
+          <t>Mizoram</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>MIP</t>
+          <t>MZM</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>140.1241112</v>
+        <v>41.0678718</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>54.8666033</v>
+        <v>0</v>
       </c>
       <c r="E25" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>54.8666033</v>
-      </c>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>Overdue Before Trigger Date</t>
+        <v>0</v>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>Current dues</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Meghalaya</t>
+          <t>Nagaland</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>MGA</t>
+          <t>NGD</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>78.0945079</v>
+        <v>65.5716819</v>
       </c>
       <c r="D26" s="6" t="n">
         <v>0</v>
@@ -1201,7 +1193,7 @@
       <c r="F26" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G26" s="10" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr">
         <is>
           <t>Current dues</t>
         </is>
@@ -1210,143 +1202,143 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Mizoram</t>
+          <t>Odisha</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>MZM</t>
+          <t>ODI</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>35.6164405</v>
+        <v>1300.287625</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>0</v>
+        <v>474.0948632</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>0</v>
+        <v>0.2621178</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="10" t="inlineStr">
-        <is>
-          <t>Current dues</t>
+        <v>474.356981</v>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Overdue After Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Nagaland</t>
+          <t>Puducherry</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>NGD</t>
+          <t>PU</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>62.5113693</v>
+        <v>290.6929106</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0</v>
+        <v>28.2946496</v>
       </c>
       <c r="E28" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="10" t="inlineStr">
-        <is>
-          <t>Current dues</t>
+        <v>28.2946496</v>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Overdue Before Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Odisha</t>
+          <t>Punjab</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>ODI</t>
+          <t>PNB</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>1672.3764556</v>
+        <v>3249.4679334</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>392.7244689</v>
+        <v>414.4290736</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>0.2621178</v>
+        <v>0</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>392.9865867</v>
-      </c>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t>Overdue After Trigger Date</t>
+        <v>414.4290736</v>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Overdue Before Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Puducherry</t>
+          <t>Rajasthan</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>PU</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>223.0331692</v>
+        <v>4382.8169765</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>0</v>
+        <v>2440.8323243</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>0</v>
+        <v>0.009858799999999999</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="10" t="inlineStr">
-        <is>
-          <t>Current dues</t>
+        <v>2440.8421831</v>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Overdue After Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Punjab</t>
+          <t>Sikkim</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>SKM</t>
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>2528.2792109</v>
+        <v>52.0196783</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>1072.5297172</v>
+        <v>31.001355</v>
       </c>
       <c r="E31" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>1072.5297172</v>
-      </c>
-      <c r="G31" s="8" t="inlineStr">
+        <v>31.001355</v>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>Overdue Before Trigger Date</t>
         </is>
@@ -1355,27 +1347,27 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Rajasthan</t>
+          <t>Tamil Nadu</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>TND</t>
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>4481.1058297</v>
+        <v>2915.8491</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>1894.1654563</v>
+        <v>849.8763079</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>0.0474065</v>
+        <v>2e-07</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>1894.2128628</v>
-      </c>
-      <c r="G32" s="9" t="inlineStr">
+        <v>849.8763081</v>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
         <is>
           <t>Overdue After Trigger Date</t>
         </is>
@@ -1384,27 +1376,27 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Sikkim</t>
+          <t>Telangana</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>SKM</t>
+          <t>TLG</t>
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>66.257171</v>
+        <v>1582.8874538</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>2.7128798</v>
+        <v>69.7638122</v>
       </c>
       <c r="E33" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>2.7128798</v>
-      </c>
-      <c r="G33" s="8" t="inlineStr">
+        <v>69.7638122</v>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
         <is>
           <t>Overdue Before Trigger Date</t>
         </is>
@@ -1413,56 +1405,56 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Tamil Nadu</t>
+          <t>Tripura</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>TND</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>3719.5318507</v>
+        <v>307.6319081</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>678.6860172</v>
+        <v>215.8977762</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>2e-07</v>
+        <v>0</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>678.6860174</v>
-      </c>
-      <c r="G34" s="9" t="inlineStr">
-        <is>
-          <t>Overdue After Trigger Date</t>
+        <v>215.8977762</v>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Overdue Before Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Telangana</t>
+          <t>Uttar Pradesh</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>TLG</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>1597.6646801</v>
+        <v>8681.8565652</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>205.6241921</v>
+        <v>5592.5716273</v>
       </c>
       <c r="E35" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>205.6241921</v>
-      </c>
-      <c r="G35" s="8" t="inlineStr">
+        <v>5592.5716273</v>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
         <is>
           <t>Overdue Before Trigger Date</t>
         </is>
@@ -1471,142 +1463,84 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Tripura</t>
+          <t>Uttarakhand</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>UTK</t>
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>320.3415829</v>
+        <v>842.2709733</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>154.7158621</v>
+        <v>143.9289141</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>0</v>
+        <v>0.2664035</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>154.7158621</v>
+        <v>144.1953176</v>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>Overdue Before Trigger Date</t>
+          <t>Overdue After Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Uttar Pradesh</t>
+          <t>West Bengal</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>BGL</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>7883.0419084</v>
+        <v>1608.4779702</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>6385.140427</v>
+        <v>189.6500489</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>0</v>
+        <v>0.3530568</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>6385.140427</v>
+        <v>190.0031057</v>
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
-          <t>Overdue Before Trigger Date</t>
+          <t>Overdue After Trigger Date</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>Uttarakhand</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>UTK</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="n">
-        <v>926.9452156999999</v>
-      </c>
-      <c r="D38" s="6" t="n">
-        <v>155.8781753</v>
-      </c>
-      <c r="E38" s="6" t="n">
-        <v>0.2634166</v>
-      </c>
-      <c r="F38" s="6" t="n">
-        <v>156.1415919</v>
-      </c>
-      <c r="G38" s="9" t="inlineStr">
-        <is>
-          <t>Overdue After Trigger Date</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>West Bengal</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>BGL</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="n">
-        <v>1920.6624006</v>
-      </c>
-      <c r="D39" s="6" t="n">
-        <v>140.554156</v>
-      </c>
-      <c r="E39" s="6" t="n">
-        <v>0.3530568</v>
-      </c>
-      <c r="F39" s="6" t="n">
-        <v>140.9072128</v>
-      </c>
-      <c r="G39" s="9" t="inlineStr">
-        <is>
-          <t>Overdue After Trigger Date</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="11" t="inlineStr">
+      <c r="A38" s="10" t="inlineStr">
         <is>
           <t>TOTAL (All India)</t>
         </is>
       </c>
-      <c r="B40" s="12" t="n"/>
-      <c r="C40" s="13" t="n">
-        <v>63071.9070643</v>
-      </c>
-      <c r="D40" s="13" t="n">
-        <v>21995.4020541</v>
-      </c>
-      <c r="E40" s="13" t="n">
-        <v>4.2842536</v>
-      </c>
-      <c r="F40" s="13" t="n">
-        <v>21999.6863077</v>
-      </c>
-      <c r="G40" s="12" t="n"/>
+      <c r="B38" s="11" t="n"/>
+      <c r="C38" s="12" t="n">
+        <v>64049.4393627</v>
+      </c>
+      <c r="D38" s="12" t="n">
+        <v>21756.8049284</v>
+      </c>
+      <c r="E38" s="12" t="n">
+        <v>4.9240963</v>
+      </c>
+      <c r="F38" s="12" t="n">
+        <v>21761.7290247</v>
+      </c>
+      <c r="G38" s="11" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G39"/>
+  <autoFilter ref="A4:G37"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>

</xml_diff>